<commit_message>
Verification workbook without data validation - plain xlsx
</commit_message>
<xml_diff>
--- a/Data Extraction/verification/model_output_verif_worklist.xlsx
+++ b/Data Extraction/verification/model_output_verif_worklist.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet name="verification" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'verification'!$A$1:$M$101</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -31,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DDE5F0"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -56,14 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -447,7 +435,7 @@
     <col width="26" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Priority</t>
@@ -566,7 +554,7 @@
         </is>
       </c>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -621,7 +609,7 @@
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -676,7 +664,7 @@
         </is>
       </c>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -731,7 +719,7 @@
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -786,7 +774,7 @@
         </is>
       </c>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -841,7 +829,7 @@
         </is>
       </c>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -896,7 +884,7 @@
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -951,7 +939,7 @@
         </is>
       </c>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -1006,7 +994,7 @@
         </is>
       </c>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -1061,7 +1049,7 @@
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -1116,7 +1104,7 @@
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -1171,7 +1159,7 @@
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -1226,7 +1214,7 @@
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
@@ -1281,7 +1269,7 @@
         </is>
       </c>
       <c r="K15" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
@@ -1336,7 +1324,7 @@
         </is>
       </c>
       <c r="K16" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1391,7 +1379,7 @@
         </is>
       </c>
       <c r="K17" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1446,7 +1434,7 @@
         </is>
       </c>
       <c r="K18" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1501,7 +1489,7 @@
         </is>
       </c>
       <c r="K19" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -1556,7 +1544,7 @@
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
@@ -1611,7 +1599,7 @@
         </is>
       </c>
       <c r="K21" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1666,7 +1654,7 @@
         </is>
       </c>
       <c r="K22" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -1721,7 +1709,7 @@
         </is>
       </c>
       <c r="K23" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -1776,7 +1764,7 @@
         </is>
       </c>
       <c r="K24" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -1831,7 +1819,7 @@
         </is>
       </c>
       <c r="K25" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -1882,7 +1870,7 @@
         </is>
       </c>
       <c r="K26" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
@@ -1937,7 +1925,7 @@
         </is>
       </c>
       <c r="K27" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
@@ -1992,7 +1980,7 @@
         </is>
       </c>
       <c r="K28" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
@@ -2047,7 +2035,7 @@
         </is>
       </c>
       <c r="K29" t="inlineStr"/>
-      <c r="L29" s="2" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
@@ -2098,7 +2086,7 @@
         </is>
       </c>
       <c r="K30" t="inlineStr"/>
-      <c r="L30" s="2" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
@@ -2153,7 +2141,7 @@
         </is>
       </c>
       <c r="K31" t="inlineStr"/>
-      <c r="L31" s="2" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
@@ -2208,7 +2196,7 @@
         </is>
       </c>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
@@ -2263,7 +2251,7 @@
         </is>
       </c>
       <c r="K33" t="inlineStr"/>
-      <c r="L33" s="2" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
@@ -2318,7 +2306,7 @@
         </is>
       </c>
       <c r="K34" t="inlineStr"/>
-      <c r="L34" s="2" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
@@ -2373,7 +2361,7 @@
         </is>
       </c>
       <c r="K35" t="inlineStr"/>
-      <c r="L35" s="2" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
@@ -2428,7 +2416,7 @@
         </is>
       </c>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" s="2" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
@@ -2483,7 +2471,7 @@
         </is>
       </c>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" s="2" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
@@ -2538,7 +2526,7 @@
         </is>
       </c>
       <c r="K38" t="inlineStr"/>
-      <c r="L38" s="2" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
@@ -2593,7 +2581,7 @@
         </is>
       </c>
       <c r="K39" t="inlineStr"/>
-      <c r="L39" s="2" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
@@ -2648,7 +2636,7 @@
         </is>
       </c>
       <c r="K40" t="inlineStr"/>
-      <c r="L40" s="2" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
@@ -2703,7 +2691,7 @@
         </is>
       </c>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" s="2" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
@@ -2758,7 +2746,7 @@
         </is>
       </c>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" s="2" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
@@ -2813,7 +2801,7 @@
         </is>
       </c>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" s="2" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
@@ -2868,7 +2856,7 @@
         </is>
       </c>
       <c r="K44" t="inlineStr"/>
-      <c r="L44" s="2" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
@@ -2923,7 +2911,7 @@
         </is>
       </c>
       <c r="K45" t="inlineStr"/>
-      <c r="L45" s="2" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
     </row>
     <row r="46">
@@ -2978,7 +2966,7 @@
         </is>
       </c>
       <c r="K46" t="inlineStr"/>
-      <c r="L46" s="2" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
@@ -3033,7 +3021,7 @@
         </is>
       </c>
       <c r="K47" t="inlineStr"/>
-      <c r="L47" s="2" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
@@ -3088,7 +3076,7 @@
         </is>
       </c>
       <c r="K48" t="inlineStr"/>
-      <c r="L48" s="2" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
@@ -3143,7 +3131,7 @@
         </is>
       </c>
       <c r="K49" t="inlineStr"/>
-      <c r="L49" s="2" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
@@ -3198,7 +3186,7 @@
         </is>
       </c>
       <c r="K50" t="inlineStr"/>
-      <c r="L50" s="2" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
@@ -3249,7 +3237,7 @@
         </is>
       </c>
       <c r="K51" t="inlineStr"/>
-      <c r="L51" s="2" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
@@ -3304,7 +3292,7 @@
         </is>
       </c>
       <c r="K52" t="inlineStr"/>
-      <c r="L52" s="2" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
@@ -3359,7 +3347,7 @@
         </is>
       </c>
       <c r="K53" t="inlineStr"/>
-      <c r="L53" s="2" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
@@ -3414,7 +3402,7 @@
         </is>
       </c>
       <c r="K54" t="inlineStr"/>
-      <c r="L54" s="2" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
@@ -3469,7 +3457,7 @@
         </is>
       </c>
       <c r="K55" t="inlineStr"/>
-      <c r="L55" s="2" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
     </row>
     <row r="56">
@@ -3524,7 +3512,7 @@
         </is>
       </c>
       <c r="K56" t="inlineStr"/>
-      <c r="L56" s="2" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
@@ -3579,7 +3567,7 @@
         </is>
       </c>
       <c r="K57" t="inlineStr"/>
-      <c r="L57" s="2" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
@@ -3634,7 +3622,7 @@
         </is>
       </c>
       <c r="K58" t="inlineStr"/>
-      <c r="L58" s="2" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr"/>
     </row>
     <row r="59">
@@ -3689,7 +3677,7 @@
         </is>
       </c>
       <c r="K59" t="inlineStr"/>
-      <c r="L59" s="2" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
@@ -3744,7 +3732,7 @@
         </is>
       </c>
       <c r="K60" t="inlineStr"/>
-      <c r="L60" s="2" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr"/>
     </row>
     <row r="61">
@@ -3799,7 +3787,7 @@
         </is>
       </c>
       <c r="K61" t="inlineStr"/>
-      <c r="L61" s="2" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
@@ -3854,7 +3842,7 @@
         </is>
       </c>
       <c r="K62" t="inlineStr"/>
-      <c r="L62" s="2" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
     </row>
     <row r="63">
@@ -3909,7 +3897,7 @@
         </is>
       </c>
       <c r="K63" t="inlineStr"/>
-      <c r="L63" s="2" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
@@ -3964,7 +3952,7 @@
         </is>
       </c>
       <c r="K64" t="inlineStr"/>
-      <c r="L64" s="2" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr"/>
     </row>
     <row r="65">
@@ -4019,7 +4007,7 @@
         </is>
       </c>
       <c r="K65" t="inlineStr"/>
-      <c r="L65" s="2" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr"/>
     </row>
     <row r="66">
@@ -4074,7 +4062,7 @@
         </is>
       </c>
       <c r="K66" t="inlineStr"/>
-      <c r="L66" s="2" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
       <c r="M66" t="inlineStr"/>
     </row>
     <row r="67">
@@ -4129,7 +4117,7 @@
         </is>
       </c>
       <c r="K67" t="inlineStr"/>
-      <c r="L67" s="2" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
       <c r="M67" t="inlineStr"/>
     </row>
     <row r="68">
@@ -4184,7 +4172,7 @@
         </is>
       </c>
       <c r="K68" t="inlineStr"/>
-      <c r="L68" s="2" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr"/>
     </row>
     <row r="69">
@@ -4239,7 +4227,7 @@
         </is>
       </c>
       <c r="K69" t="inlineStr"/>
-      <c r="L69" s="2" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
       <c r="M69" t="inlineStr"/>
     </row>
     <row r="70">
@@ -4294,7 +4282,7 @@
         </is>
       </c>
       <c r="K70" t="inlineStr"/>
-      <c r="L70" s="2" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
       <c r="M70" t="inlineStr"/>
     </row>
     <row r="71">
@@ -4349,7 +4337,7 @@
         </is>
       </c>
       <c r="K71" t="inlineStr"/>
-      <c r="L71" s="2" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
       <c r="M71" t="inlineStr"/>
     </row>
     <row r="72">
@@ -4404,7 +4392,7 @@
         </is>
       </c>
       <c r="K72" t="inlineStr"/>
-      <c r="L72" s="2" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
       <c r="M72" t="inlineStr"/>
     </row>
     <row r="73">
@@ -4459,7 +4447,7 @@
         </is>
       </c>
       <c r="K73" t="inlineStr"/>
-      <c r="L73" s="2" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
       <c r="M73" t="inlineStr"/>
     </row>
     <row r="74">
@@ -4514,7 +4502,7 @@
         </is>
       </c>
       <c r="K74" t="inlineStr"/>
-      <c r="L74" s="2" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr"/>
     </row>
     <row r="75">
@@ -4569,7 +4557,7 @@
         </is>
       </c>
       <c r="K75" t="inlineStr"/>
-      <c r="L75" s="2" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
       <c r="M75" t="inlineStr"/>
     </row>
     <row r="76">
@@ -4624,7 +4612,7 @@
         </is>
       </c>
       <c r="K76" t="inlineStr"/>
-      <c r="L76" s="2" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr"/>
     </row>
     <row r="77">
@@ -4679,7 +4667,7 @@
         </is>
       </c>
       <c r="K77" t="inlineStr"/>
-      <c r="L77" s="2" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
       <c r="M77" t="inlineStr"/>
     </row>
     <row r="78">
@@ -4734,7 +4722,7 @@
         </is>
       </c>
       <c r="K78" t="inlineStr"/>
-      <c r="L78" s="2" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr"/>
     </row>
     <row r="79">
@@ -4789,7 +4777,7 @@
         </is>
       </c>
       <c r="K79" t="inlineStr"/>
-      <c r="L79" s="2" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
       <c r="M79" t="inlineStr"/>
     </row>
     <row r="80">
@@ -4844,7 +4832,7 @@
         </is>
       </c>
       <c r="K80" t="inlineStr"/>
-      <c r="L80" s="2" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
       <c r="M80" t="inlineStr"/>
     </row>
     <row r="81">
@@ -4899,7 +4887,7 @@
         </is>
       </c>
       <c r="K81" t="inlineStr"/>
-      <c r="L81" s="2" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr"/>
     </row>
     <row r="82">
@@ -4954,7 +4942,7 @@
         </is>
       </c>
       <c r="K82" t="inlineStr"/>
-      <c r="L82" s="2" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
       <c r="M82" t="inlineStr"/>
     </row>
     <row r="83">
@@ -5009,7 +4997,7 @@
         </is>
       </c>
       <c r="K83" t="inlineStr"/>
-      <c r="L83" s="2" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
       <c r="M83" t="inlineStr"/>
     </row>
     <row r="84">
@@ -5064,7 +5052,7 @@
         </is>
       </c>
       <c r="K84" t="inlineStr"/>
-      <c r="L84" s="2" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
       <c r="M84" t="inlineStr"/>
     </row>
     <row r="85">
@@ -5119,7 +5107,7 @@
         </is>
       </c>
       <c r="K85" t="inlineStr"/>
-      <c r="L85" s="2" t="inlineStr"/>
+      <c r="L85" t="inlineStr"/>
       <c r="M85" t="inlineStr"/>
     </row>
     <row r="86">
@@ -5174,7 +5162,7 @@
         </is>
       </c>
       <c r="K86" t="inlineStr"/>
-      <c r="L86" s="2" t="inlineStr"/>
+      <c r="L86" t="inlineStr"/>
       <c r="M86" t="inlineStr"/>
     </row>
     <row r="87">
@@ -5229,7 +5217,7 @@
         </is>
       </c>
       <c r="K87" t="inlineStr"/>
-      <c r="L87" s="2" t="inlineStr"/>
+      <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr"/>
     </row>
     <row r="88">
@@ -5284,7 +5272,7 @@
         </is>
       </c>
       <c r="K88" t="inlineStr"/>
-      <c r="L88" s="2" t="inlineStr"/>
+      <c r="L88" t="inlineStr"/>
       <c r="M88" t="inlineStr"/>
     </row>
     <row r="89">
@@ -5339,7 +5327,7 @@
         </is>
       </c>
       <c r="K89" t="inlineStr"/>
-      <c r="L89" s="2" t="inlineStr"/>
+      <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr"/>
     </row>
     <row r="90">
@@ -5394,7 +5382,7 @@
         </is>
       </c>
       <c r="K90" t="inlineStr"/>
-      <c r="L90" s="2" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr"/>
     </row>
     <row r="91">
@@ -5449,7 +5437,7 @@
         </is>
       </c>
       <c r="K91" t="inlineStr"/>
-      <c r="L91" s="2" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr"/>
     </row>
     <row r="92">
@@ -5504,7 +5492,7 @@
         </is>
       </c>
       <c r="K92" t="inlineStr"/>
-      <c r="L92" s="2" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
       <c r="M92" t="inlineStr"/>
     </row>
     <row r="93">
@@ -5559,7 +5547,7 @@
         </is>
       </c>
       <c r="K93" t="inlineStr"/>
-      <c r="L93" s="2" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr"/>
     </row>
     <row r="94">
@@ -5614,7 +5602,7 @@
         </is>
       </c>
       <c r="K94" t="inlineStr"/>
-      <c r="L94" s="2" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr"/>
     </row>
     <row r="95">
@@ -5669,7 +5657,7 @@
         </is>
       </c>
       <c r="K95" t="inlineStr"/>
-      <c r="L95" s="2" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
       <c r="M95" t="inlineStr"/>
     </row>
     <row r="96">
@@ -5724,7 +5712,7 @@
         </is>
       </c>
       <c r="K96" t="inlineStr"/>
-      <c r="L96" s="2" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
       <c r="M96" t="inlineStr"/>
     </row>
     <row r="97">
@@ -5775,7 +5763,7 @@
         </is>
       </c>
       <c r="K97" t="inlineStr"/>
-      <c r="L97" s="2" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr"/>
     </row>
     <row r="98">
@@ -5830,7 +5818,7 @@
         </is>
       </c>
       <c r="K98" t="inlineStr"/>
-      <c r="L98" s="2" t="inlineStr"/>
+      <c r="L98" t="inlineStr"/>
       <c r="M98" t="inlineStr"/>
     </row>
     <row r="99">
@@ -5885,7 +5873,7 @@
         </is>
       </c>
       <c r="K99" t="inlineStr"/>
-      <c r="L99" s="2" t="inlineStr"/>
+      <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr"/>
     </row>
     <row r="100">
@@ -5940,7 +5928,7 @@
         </is>
       </c>
       <c r="K100" t="inlineStr"/>
-      <c r="L100" s="2" t="inlineStr"/>
+      <c r="L100" t="inlineStr"/>
       <c r="M100" t="inlineStr"/>
     </row>
     <row r="101">
@@ -5995,16 +5983,10 @@
         </is>
       </c>
       <c r="K101" t="inlineStr"/>
-      <c r="L101" s="2" t="inlineStr"/>
+      <c r="L101" t="inlineStr"/>
       <c r="M101" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M101"/>
-  <dataValidations count="1">
-    <dataValidation sqref="K2:K101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Pick one" error="Choose one of the seven options." promptTitle="Is the extraction correct?" prompt="Correct = matches the PDF. Wrong numbers = a value misread. Wrong table = wrong exhibit used. Wrong method = values right, calculation wrong. Image = table is a picture. Not in PDF = not published. Question = needs a methodology decision (don't decide it)." type="list">
-      <formula1>"Correct,Wrong numbers,Wrong table,Wrong method,Image,Not in PDF,Question"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6292,13 +6274,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6B01C19-01E0-41D2-813E-A57DEA321648}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A03A84B-0B0C-4A2E-8492-149A72768352}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{78FF1695-F79E-4EA2-852A-7A2340419314}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20630461-4458-44BE-AA4B-54A5C230FEF0}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80962F69-1C0B-48F6-9145-FB0359D8CB14}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1011D01F-DA10-4ACA-8DAC-3637BBB2A22F}"/>
 </file>
</xml_diff>